<commit_message>
update the auto generate yaml file
</commit_message>
<xml_diff>
--- a/data/raw/RPi_Pico_W_Official.xlsx
+++ b/data/raw/RPi_Pico_W_Official.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\szb75\Documents\Other_Proj\ArchitecturalCarbonModelingTool\ACT\data\raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DC9985C2-EA95-4101-B8EA-E4D1DDE0C426}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5F31162F-D9A2-4DB9-8C92-A6A2116C1894}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="11500" xr2:uid="{EFECAB25-8862-4039-872A-9D66B4D0B167}"/>
+    <workbookView xWindow="-120" yWindow="-18120" windowWidth="29040" windowHeight="17520" xr2:uid="{EFECAB25-8862-4039-872A-9D66B4D0B167}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>

</xml_diff>